<commit_message>
init: proyecto herramientas financieras AR
</commit_message>
<xml_diff>
--- a/lecaps_datos_estaticos.xlsx
+++ b/lecaps_datos_estaticos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IA\Dashboard_Financiero\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{03061B5A-B822-4C70-A576-0F4A82A8B28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4676655-1FDD-4DDC-B36E-5E8B61952A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Instrucciones" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="104">
   <si>
     <t>HERRAMIENTAS FINANCIERAS AR — Datos Estáticos de Instrumentos</t>
   </si>
@@ -347,6 +346,18 @@
   </si>
   <si>
     <t>NO PAGA</t>
+  </si>
+  <si>
+    <t>S17L6</t>
+  </si>
+  <si>
+    <t>2026-07-17</t>
+  </si>
+  <si>
+    <t>S14G6</t>
+  </si>
+  <si>
+    <t>2026-08-14</t>
   </si>
 </sst>
 </file>
@@ -357,7 +368,7 @@
     <numFmt numFmtId="164" formatCode="0.00&quot;%&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000&quot;%&quot;"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -446,6 +457,19 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFF0F2F5"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -497,7 +521,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -571,6 +595,12 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -581,7 +611,13 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -908,7 +944,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -919,38 +955,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
+      <c r="A1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
     </row>
     <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
     </row>
     <row r="4" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -1041,41 +1077,41 @@
       <c r="B6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="28">
+      <c r="D6" s="25">
         <v>1.1012999999999999</v>
       </c>
-      <c r="E6" s="28">
+      <c r="E6" s="25">
         <v>1.0034000000000001</v>
       </c>
-      <c r="F6" s="28">
+      <c r="F6" s="25">
         <v>0.08</v>
       </c>
-      <c r="G6" s="28">
+      <c r="G6" s="25">
         <v>1.0032000000000001</v>
       </c>
-      <c r="H6" s="28" t="s">
+      <c r="H6" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="I6" s="28">
+      <c r="I6" s="25">
         <v>0</v>
       </c>
       <c r="J6" s="7">
-        <f t="shared" ref="J6:J19" ca="1" si="0">MAX(0,INT(DATE(LEFT(C6,4),MID(C6,6,2),RIGHT(C6,2))-TODAY()))</f>
+        <f t="shared" ref="J6:J21" ca="1" si="0">MAX(0,INT(DATE(LEFT(C6,4),MID(C6,6,2),RIGHT(C6,2))-TODAY()))</f>
         <v>0</v>
       </c>
       <c r="K6" s="8" t="str">
-        <f t="shared" ref="K6:K19" ca="1" si="1">IF(J6&gt;0,((D6/D6)^(365/J6)-1)*100,"—")</f>
+        <f t="shared" ref="K6:K21" ca="1" si="1">IF(J6&gt;0,((D6/D6)^(365/J6)-1)*100,"—")</f>
         <v>—</v>
       </c>
       <c r="L6" s="8" t="str">
-        <f t="shared" ref="L6:L19" ca="1" si="2">IF(J6&gt;0,(D6/D6-1)*(365/J6)*100,"—")</f>
+        <f t="shared" ref="L6:L21" ca="1" si="2">IF(J6&gt;0,(D6/D6-1)*(365/J6)*100,"—")</f>
         <v>—</v>
       </c>
       <c r="M6" s="9" t="str">
-        <f t="shared" ref="M6:M19" ca="1" si="3">IF(J6&gt;0,((D6/D6)^(30/J6)-1)*100,"—")</f>
+        <f t="shared" ref="M6:M21" ca="1" si="3">IF(J6&gt;0,((D6/D6)^(30/J6)-1)*100,"—")</f>
         <v>—</v>
       </c>
     </row>
@@ -1086,30 +1122,30 @@
       <c r="B7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="26">
         <v>1.2748600000000001</v>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="26">
         <v>1.0235000000000001</v>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="26">
         <v>0.22</v>
       </c>
-      <c r="G7" s="29">
+      <c r="G7" s="26">
         <v>1.0193000000000001</v>
       </c>
-      <c r="H7" s="29" t="s">
+      <c r="H7" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I7" s="29">
+      <c r="I7" s="26">
         <v>0</v>
       </c>
       <c r="J7" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K7" s="13">
         <f t="shared" ca="1" si="1"/>
@@ -1131,30 +1167,30 @@
       <c r="B8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="29">
+      <c r="D8" s="26">
         <v>1.0517799999999999</v>
       </c>
-      <c r="E8" s="28">
+      <c r="E8" s="25">
         <v>1.0069999999999999</v>
       </c>
-      <c r="F8" s="28">
+      <c r="F8" s="25">
         <v>0.01</v>
       </c>
-      <c r="G8" s="28">
+      <c r="G8" s="25">
         <v>1.0069999999999999</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="H8" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I8" s="29">
+      <c r="I8" s="26">
         <v>0</v>
       </c>
       <c r="J8" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K8" s="8">
         <f t="shared" ca="1" si="1"/>
@@ -1176,30 +1212,30 @@
       <c r="B9" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="26">
         <v>1.3204400000000001</v>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="26">
         <v>1.0063</v>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="26">
         <v>0.25</v>
       </c>
-      <c r="G9" s="29">
+      <c r="G9" s="26">
         <v>1.0049999999999999</v>
       </c>
-      <c r="H9" s="29" t="s">
+      <c r="H9" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I9" s="29">
+      <c r="I9" s="26">
         <v>0</v>
       </c>
       <c r="J9" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K9" s="13">
         <f t="shared" ca="1" si="1"/>
@@ -1221,30 +1257,30 @@
       <c r="B10" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="25">
         <v>1.44896</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="25">
         <v>0.99399999999999999</v>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="25">
         <v>0.35</v>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="25">
         <v>0.99550000000000005</v>
       </c>
-      <c r="H10" s="29" t="s">
+      <c r="H10" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I10" s="29">
+      <c r="I10" s="26">
         <v>0</v>
       </c>
       <c r="J10" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K10" s="8">
         <f t="shared" ca="1" si="1"/>
@@ -1260,171 +1296,171 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
-        <v>37</v>
+      <c r="A11" s="31" t="s">
+        <v>100</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" s="26">
+        <v>1.1767700000000001</v>
+      </c>
+      <c r="E11" s="26">
+        <v>1.0219</v>
+      </c>
+      <c r="F11" s="26">
+        <v>0.05</v>
+      </c>
+      <c r="G11" s="26">
+        <v>1.0208999999999999</v>
+      </c>
+      <c r="H11" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="I11" s="26">
+        <v>0</v>
+      </c>
+      <c r="J11" s="7">
+        <f t="shared" ca="1" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="K11" s="13">
+        <f t="shared" ref="K11" ca="1" si="4">IF(J11&gt;0,((D11/D11)^(365/J11)-1)*100,"—")</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="13">
+        <f t="shared" ref="L11" ca="1" si="5">IF(J11&gt;0,(D11/D11-1)*(365/J11)*100,"—")</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="14">
+        <f t="shared" ref="M11" ca="1" si="6">IF(J11&gt;0,((D11/D11)^(30/J11)-1)*100,"—")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="29">
+      <c r="D12" s="26">
         <v>1.1767700000000001</v>
       </c>
-      <c r="E11" s="29">
+      <c r="E12" s="26">
         <v>1.0219</v>
       </c>
-      <c r="F11" s="29">
+      <c r="F12" s="26">
         <v>0.05</v>
       </c>
-      <c r="G11" s="29">
+      <c r="G12" s="26">
         <v>1.0208999999999999</v>
       </c>
-      <c r="H11" s="29" t="s">
+      <c r="H12" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I11" s="29">
-        <v>0</v>
-      </c>
-      <c r="J11" s="12">
+      <c r="I12" s="26">
+        <v>0</v>
+      </c>
+      <c r="J12" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>105</v>
-      </c>
-      <c r="K11" s="13">
+        <v>104</v>
+      </c>
+      <c r="K12" s="13">
         <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
-      <c r="L11" s="13">
+      <c r="L12" s="13">
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="M11" s="14">
+      <c r="M12" s="14">
         <f t="shared" ca="1" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="6" t="s">
+    <row r="13" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="33" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="28">
+      <c r="C13" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="D13" s="30">
         <v>1.27064</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E13" s="30">
         <v>1.0163</v>
       </c>
-      <c r="F12" s="28">
+      <c r="F13" s="30">
         <v>0.12</v>
       </c>
-      <c r="G12" s="28">
+      <c r="G13" s="30">
         <v>1.0145999999999999</v>
       </c>
-      <c r="H12" s="29" t="s">
+      <c r="H13" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I12" s="29">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7">
-        <f t="shared" ca="1" si="0"/>
-        <v>136</v>
-      </c>
-      <c r="K12" s="8">
-        <f t="shared" ca="1" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="L12" s="8">
-        <f t="shared" ca="1" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M12" s="9">
-        <f t="shared" ca="1" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="28">
-        <v>1.17536</v>
-      </c>
-      <c r="E13" s="29">
-        <v>1.0132000000000001</v>
-      </c>
-      <c r="F13" s="29">
-        <v>0.01</v>
-      </c>
-      <c r="G13" s="29">
-        <v>1.0130999999999999</v>
-      </c>
-      <c r="H13" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="I13" s="29">
-        <v>0</v>
-      </c>
-      <c r="J13" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>166</v>
-      </c>
-      <c r="K13" s="13">
-        <f t="shared" ca="1" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="L13" s="13">
-        <f t="shared" ca="1" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M13" s="14">
-        <f t="shared" ca="1" si="3"/>
+      <c r="I13" s="26">
+        <v>0</v>
+      </c>
+      <c r="J13" s="7">
+        <f t="shared" ref="J13" ca="1" si="7">MAX(0,INT(DATE(LEFT(C13,4),MID(C13,6,2),RIGHT(C13,2))-TODAY()))</f>
+        <v>118</v>
+      </c>
+      <c r="K13" s="8">
+        <f t="shared" ref="K13" ca="1" si="8">IF(J13&gt;0,((D13/D13)^(365/J13)-1)*100,"—")</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="8">
+        <f t="shared" ref="L13" ca="1" si="9">IF(J13&gt;0,(D13/D13-1)*(365/J13)*100,"—")</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="9">
+        <f t="shared" ref="M13" ca="1" si="10">IF(J13&gt;0,((D13/D13)^(30/J13)-1)*100,"—")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="28">
-        <v>1.3527800000000001</v>
-      </c>
-      <c r="E14" s="28">
-        <v>1.1487000000000001</v>
-      </c>
-      <c r="F14" s="28">
-        <v>0</v>
-      </c>
-      <c r="G14" s="28">
-        <v>1.1487000000000001</v>
-      </c>
-      <c r="H14" s="29" t="s">
+      <c r="C14" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="25">
+        <v>1.27064</v>
+      </c>
+      <c r="E14" s="25">
+        <v>1.0163</v>
+      </c>
+      <c r="F14" s="25">
+        <v>0.12</v>
+      </c>
+      <c r="G14" s="25">
+        <v>1.0145999999999999</v>
+      </c>
+      <c r="H14" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I14" s="29">
+      <c r="I14" s="26">
         <v>0</v>
       </c>
       <c r="J14" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>196</v>
+        <v>135</v>
       </c>
       <c r="K14" s="8">
         <f t="shared" ca="1" si="1"/>
@@ -1441,35 +1477,35 @@
     </row>
     <row r="15" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="29">
-        <v>1.29888</v>
-      </c>
-      <c r="E15" s="29">
-        <v>1.0740000000000001</v>
-      </c>
-      <c r="F15" s="29">
-        <v>0</v>
-      </c>
-      <c r="G15" s="29">
-        <v>1.0740000000000001</v>
-      </c>
-      <c r="H15" s="29" t="s">
+      <c r="C15" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="25">
+        <v>1.17536</v>
+      </c>
+      <c r="E15" s="26">
+        <v>1.0132000000000001</v>
+      </c>
+      <c r="F15" s="26">
+        <v>0.01</v>
+      </c>
+      <c r="G15" s="26">
+        <v>1.0130999999999999</v>
+      </c>
+      <c r="H15" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I15" s="29">
+      <c r="I15" s="26">
         <v>0</v>
       </c>
       <c r="J15" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>227</v>
+        <v>165</v>
       </c>
       <c r="K15" s="13">
         <f t="shared" ca="1" si="1"/>
@@ -1486,35 +1522,35 @@
     </row>
     <row r="16" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="28">
-        <v>1.61104</v>
-      </c>
-      <c r="E16" s="28">
-        <v>0.95920000000000005</v>
-      </c>
-      <c r="F16" s="28">
-        <v>0.32</v>
-      </c>
-      <c r="G16" s="28">
-        <v>0.96919999999999995</v>
-      </c>
-      <c r="H16" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="25">
+        <v>1.3527800000000001</v>
+      </c>
+      <c r="E16" s="25">
+        <v>1.1487000000000001</v>
+      </c>
+      <c r="F16" s="25">
+        <v>0</v>
+      </c>
+      <c r="G16" s="25">
+        <v>1.1487000000000001</v>
+      </c>
+      <c r="H16" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I16" s="29">
+      <c r="I16" s="26">
         <v>0</v>
       </c>
       <c r="J16" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>273</v>
+        <v>195</v>
       </c>
       <c r="K16" s="8">
         <f t="shared" ca="1" si="1"/>
@@ -1531,35 +1567,35 @@
     </row>
     <row r="17" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="D17" s="29">
-        <v>1.57341</v>
-      </c>
-      <c r="E17" s="29">
-        <v>1.1625000000000001</v>
-      </c>
-      <c r="F17" s="29">
-        <v>0</v>
-      </c>
-      <c r="G17" s="29">
-        <v>1.1625000000000001</v>
-      </c>
-      <c r="H17" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="26">
+        <v>1.29888</v>
+      </c>
+      <c r="E17" s="26">
+        <v>1.0740000000000001</v>
+      </c>
+      <c r="F17" s="26">
+        <v>0</v>
+      </c>
+      <c r="G17" s="26">
+        <v>1.0740000000000001</v>
+      </c>
+      <c r="H17" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I17" s="29">
+      <c r="I17" s="26">
         <v>0</v>
       </c>
       <c r="J17" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>378</v>
+        <v>226</v>
       </c>
       <c r="K17" s="13">
         <f t="shared" ca="1" si="1"/>
@@ -1576,35 +1612,35 @@
     </row>
     <row r="18" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="28">
-        <v>1.51563</v>
-      </c>
-      <c r="E18" s="28">
-        <v>1.0920000000000001</v>
-      </c>
-      <c r="F18" s="28">
-        <v>0</v>
-      </c>
-      <c r="G18" s="28">
-        <v>1.0920000000000001</v>
-      </c>
-      <c r="H18" s="29" t="s">
+      <c r="C18" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="25">
+        <v>1.61104</v>
+      </c>
+      <c r="E18" s="25">
+        <v>0.95920000000000005</v>
+      </c>
+      <c r="F18" s="25">
+        <v>0.32</v>
+      </c>
+      <c r="G18" s="25">
+        <v>0.96919999999999995</v>
+      </c>
+      <c r="H18" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I18" s="29">
+      <c r="I18" s="26">
         <v>0</v>
       </c>
       <c r="J18" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>409</v>
+        <v>272</v>
       </c>
       <c r="K18" s="8">
         <f t="shared" ca="1" si="1"/>
@@ -1621,35 +1657,35 @@
     </row>
     <row r="19" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B19" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="29">
-        <v>1.56037</v>
-      </c>
-      <c r="E19" s="29">
-        <v>1.0465</v>
-      </c>
-      <c r="F19" s="29">
-        <v>0.06</v>
-      </c>
-      <c r="G19" s="29">
-        <v>1.0439000000000001</v>
-      </c>
-      <c r="H19" s="29" t="s">
+      <c r="C19" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="26">
+        <v>1.57341</v>
+      </c>
+      <c r="E19" s="26">
+        <v>1.1625000000000001</v>
+      </c>
+      <c r="F19" s="26">
+        <v>0</v>
+      </c>
+      <c r="G19" s="26">
+        <v>1.1625000000000001</v>
+      </c>
+      <c r="H19" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="I19" s="29">
+      <c r="I19" s="26">
         <v>0</v>
       </c>
       <c r="J19" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>439</v>
+        <v>377</v>
       </c>
       <c r="K19" s="13">
         <f t="shared" ca="1" si="1"/>
@@ -1660,6 +1696,96 @@
         <v>0</v>
       </c>
       <c r="M19" s="14">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="25">
+        <v>1.51563</v>
+      </c>
+      <c r="E20" s="25">
+        <v>1.0920000000000001</v>
+      </c>
+      <c r="F20" s="25">
+        <v>0</v>
+      </c>
+      <c r="G20" s="25">
+        <v>1.0920000000000001</v>
+      </c>
+      <c r="H20" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="I20" s="26">
+        <v>0</v>
+      </c>
+      <c r="J20" s="7">
+        <f t="shared" ca="1" si="0"/>
+        <v>408</v>
+      </c>
+      <c r="K20" s="8">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L20" s="8">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M20" s="9">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="26">
+        <v>1.56037</v>
+      </c>
+      <c r="E21" s="26">
+        <v>1.0465</v>
+      </c>
+      <c r="F21" s="26">
+        <v>0.06</v>
+      </c>
+      <c r="G21" s="26">
+        <v>1.0439000000000001</v>
+      </c>
+      <c r="H21" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="I21" s="26">
+        <v>0</v>
+      </c>
+      <c r="J21" s="12">
+        <f t="shared" ca="1" si="0"/>
+        <v>438</v>
+      </c>
+      <c r="K21" s="13">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L21" s="13">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M21" s="14">
         <f t="shared" ca="1" si="3"/>
         <v>0</v>
       </c>
@@ -1669,6 +1795,7 @@
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
+  <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>